<commit_message>
Actualizar cierre Menendez Pidal: ingresos agosto y Obramat
</commit_message>
<xml_diff>
--- a/tabla_maestra_irpf_2025_menendez_pidal.xlsx
+++ b/tabla_maestra_irpf_2025_menendez_pidal.xlsx
@@ -2186,230 +2186,296 @@
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr" s="1">
-        <is>
-          <t>ejercicio_devengo</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr" s="1">
-        <is>
-          <t>riesgo_o_pendiente</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr" s="1">
-        <is>
-          <t>nivel</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr" s="1">
-        <is>
-          <t>accion_recomendada</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>ITP aplicado con beneficio vivienda habitual</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Alto</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Revisar coherencia con destino real posterior y narrativa documental</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Contratos Antonio Cano</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Alto</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Revisar encaje documental y efecto en ingresos/ocupación</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Calificación reparación vs mejora</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Alto</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Separar con criterio técnico-fiscal porque cambia deducción/amortización</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Dependencia de lo declarado en 2023/2024</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Alto</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>La estrategia 2025 debe ser coherente con años previos</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Seguro declarado como residencia habitual</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Medio</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Revisar coherencia con alquiler por habitaciones</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Superficie seguro 98 m2 vs 81,48 m2 registrales/catastrales</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Medio</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Corregir en próxima renovación si procede</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Importes OBRAMAT ya extraídos pero falta clasificación técnica</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Medio</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Resolver reparación vs mejora antes del cierre definitivo</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Tickets IKEA simplificados flojos</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Medio-Alto</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Intentar factura nominativa o dejarlos fuera</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Falta nota simple actualizada postcompra</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Bajo</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>No bloquea IRPF 2025, pero redondea expediente</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-</worksheet>
+<ns0:worksheet xmlns:ns0="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <ns0:sheetData>
+    <ns0:row r="1">
+      <ns0:c r="A1" t="inlineStr" s="1">
+        <ns0:is>
+          <ns0:t>ejercicio_devengo</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B1" t="inlineStr" s="1">
+        <ns0:is>
+          <ns0:t>riesgo_o_pendiente</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C1" t="inlineStr" s="1">
+        <ns0:is>
+          <ns0:t>nivel</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D1" t="inlineStr" s="1">
+        <ns0:is>
+          <ns0:t>accion_recomendada</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="2">
+      <ns0:c r="A2" t="inlineStr">
+        <ns0:is>
+          <ns0:t>2025</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B2" t="inlineStr">
+        <ns0:is>
+          <ns0:t>ITP aplicado con beneficio vivienda habitual</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C2" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Alto</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D2" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Revisar coherencia con destino real posterior y narrativa documental</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="3">
+      <ns0:c r="A3" t="inlineStr">
+        <ns0:is>
+          <ns0:t>2025</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B3" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Contratos Antonio Cano</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C3" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Alto</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D3" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Revisar encaje documental y efecto en ingresos/ocupación</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="4">
+      <ns0:c r="A4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>2025</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Calificación reparación vs mejora</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Alto</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Separar con criterio técnico-fiscal porque cambia deducción/amortización</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="5">
+      <ns0:c r="A5" t="inlineStr">
+        <ns0:is>
+          <ns0:t>2025</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B5" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Dependencia de lo declarado en 2023/2024</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C5" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Alto</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D5" t="inlineStr">
+        <ns0:is>
+          <ns0:t>La estrategia 2025 debe ser coherente con años previos</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="6">
+      <ns0:c r="A6" t="inlineStr">
+        <ns0:is>
+          <ns0:t>2025</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B6" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Seguro declarado como residencia habitual</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C6" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Medio</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D6" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Revisar coherencia con alquiler por habitaciones</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="7">
+      <ns0:c r="A7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>2025</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Superficie seguro 98 m2 vs 81,48 m2 registrales/catastrales</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Medio</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Corregir en próxima renovación si procede</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="8">
+      <ns0:c r="A8" t="inlineStr">
+        <ns0:is>
+          <ns0:t>2025</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B8" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Importes OBRAMAT ya extraídos pero falta clasificación técnica</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C8" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Medio</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D8" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Resolver reparación vs mejora antes del cierre definitivo</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="9">
+      <ns0:c r="A9" t="inlineStr">
+        <ns0:is>
+          <ns0:t>2025</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B9" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Tickets IKEA simplificados flojos</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C9" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Medio-Alto</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D9" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Intentar factura nominativa o dejarlos fuera</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="10">
+      <ns0:c r="A10" t="inlineStr">
+        <ns0:is>
+          <ns0:t>2025</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B10" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Falta nota simple actualizada postcompra</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C10" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Bajo</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D10" t="inlineStr">
+        <ns0:is>
+          <ns0:t>No bloquea IRPF 2025, pero redondea expediente</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="11">
+      <ns0:c r="A11" t="inlineStr">
+        <ns0:is>
+          <ns0:t>2025</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B11" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Ingreso puntual no recurrente (fianza + arranque agosto con mediación)</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C11" t="inlineStr">
+        <ns0:is>
+          <ns0:t>MEDIO</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D11" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Jero aclaró que los 1.412 € se leen como 1.200 € de fianza + 212 € de ingreso real para él, con 600 € absorbidos por la inmobiliaria por medio mes de gestión. Mantener 212 € como ingreso inicial de Jero y dejar septiembre como transición no del todo cerrada por habitación.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="12">
+      <ns0:c r="A12" t="inlineStr">
+        <ns0:is>
+          <ns0:t>2025</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B12" t="inlineStr">
+        <ns0:is>
+          <ns0:t>OBRAMAT: anticipos 398765, 404208, 421861 y 436986 localizados</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C12" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Medio</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D12" t="inlineStr">
+        <ns0:is>
+          <ns0:t>No sumarlos además de las facturas de entrega, porque replican el mismo TTI de los pedidos 228131, 228543, 229407 y 230379; usarlos como refuerzo documental y trazabilidad de pago.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="13">
+      <ns0:c r="A13" t="inlineStr">
+        <ns0:is>
+          <ns0:t>2025</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B13" t="inlineStr">
+        <ns0:is>
+          <ns0:t>OBRAMAT: compras adicionales omitidas ya localizadas parcialmente</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C13" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Medio</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D13" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Valorar incorporación separada de 404213 (80,19 €), 407792 (21,90 €), 452497 (39,53 €) y 452516 (135,00 €). Falta concretar si existe quinta omitida adicional o si el conteo del usuario incluía también el anticipo 404208.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+  </ns0:sheetData>
+</ns0:worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3244,1250 +3310,1746 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr" s="1">
-        <is>
-          <t>ejercicio_devengo</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr" s="1">
-        <is>
-          <t>fecha</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr" s="1">
-        <is>
-          <t>proveedor</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr" s="1">
-        <is>
-          <t>bloque</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr" s="1">
-        <is>
-          <t>subbloque</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr" s="1">
-        <is>
-          <t>concepto</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr" s="1">
-        <is>
-          <t>documento</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr" s="1">
-        <is>
-          <t>pedido_o_ref</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr" s="1">
-        <is>
-          <t>importe_total_eur</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr" s="1">
-        <is>
-          <t>usar_hacienda</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr" s="1">
-        <is>
-          <t>nivel_soporte</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr" s="1">
-        <is>
-          <t>observaciones</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>2023</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>2023-11-28</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>OBRAMAT</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>reforma</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>obra_reforma</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Materiales reforma pedido 228131</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Factura 003-0011-399514</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>228131</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>4803.37</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>FUERTE</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>Factura duplicada con titular NIF y direccion de Menendez Pidal; importe total TTI extraído por pdftotext de factura PDF</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>2023</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>2023-12-07</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>OBRAMAT</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>reforma</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>obra_reforma</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Materiales reforma pedido 228543</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Factura 003-0012-404381</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>228543</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>161.13</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>FUERTE</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>Factura duplicada con titular NIF y direccion de Menendez Pidal; importe total TTI extraído por pdftotext de factura PDF</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>2024</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>2024-01-17</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>OBRAMAT</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>reforma</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>obra_reforma</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Materiales reforma pedido 229407</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Factura 003-0001-424413</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>229407</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>1037.22</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>FUERTE</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>Factura duplicada con titular NIF y direccion de Menendez Pidal; importe total TTI extraído por pdftotext de factura PDF</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>2024</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>2024-02-08</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>OBRAMAT</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>reforma</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>obra_reforma</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>Materiales reforma pedido 230379</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>Factura 003-0002-437264</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>230379</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>150.37</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>FUERTE</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>Factura duplicada con titular NIF y direccion de Menendez Pidal; importe total TTI extraído por pdftotext de factura PDF</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>2024</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>2024-04-15</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>CECOTEC</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>reforma</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>equipamiento_fijo</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>Frigorifico Bolero CoolMarket Combi 250 White E</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>Factura 259006389</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>256CEC-259006389</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>329.00</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>FUERTE</t>
-        </is>
-      </c>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>Factura nominativa sustitutiva de simplificada; facturas sustitutivas/canje emitidas el 08/06/2026 para compras de 2024, conservar tickets originales</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>2024</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>2024-04-19</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>CECOTEC</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>mobiliario</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>mobiliario_y_equipamiento</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>Colchon Flow Viscocare 1900 120x190 unidad 1</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>Factura 259006390</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>256CEC-259006390</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>119.00</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>FUERTE</t>
-        </is>
-      </c>
-      <c r="L7" t="inlineStr">
-        <is>
-          <t>Factura nominativa sustitutiva de simplificada; facturas sustitutivas/canje emitidas el 08/06/2026 para compras de 2024, conservar tickets originales</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>2024</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>2024-04-19</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>CECOTEC</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>mobiliario</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>mobiliario_y_equipamiento</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>Colchon Flow Viscocare 1900 120x190 unidad 2</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>Factura 259006391</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>256CEC-259006391</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>119.00</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>FUERTE</t>
-        </is>
-      </c>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t>Factura nominativa sustitutiva de simplificada; facturas sustitutivas/canje emitidas el 08/06/2026 para compras de 2024, conservar tickets originales</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>2024</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>2024-04-19</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>CECOTEC</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>mobiliario</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>mobiliario_y_equipamiento</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>Colchon Flow Viscocare 1900 120x190 unidad 3</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>Factura 259006392</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>256CEC-259006392</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>119.00</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>FUERTE</t>
-        </is>
-      </c>
-      <c r="L9" t="inlineStr">
-        <is>
-          <t>Factura nominativa sustitutiva de simplificada; facturas sustitutivas/canje emitidas el 08/06/2026 para compras de 2024, conservar tickets originales</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>2024</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>2024-04-19</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>CECOTEC</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>mobiliario</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>mobiliario_y_equipamiento</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>Colchon Flow Viscocare 1900 120x190 unidad 4</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>Factura 259006393</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>256CEC-259006393</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>119.00</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>FUERTE</t>
-        </is>
-      </c>
-      <c r="L10" t="inlineStr">
-        <is>
-          <t>Factura nominativa sustitutiva de simplificada; facturas sustitutivas/canje emitidas el 08/06/2026 para compras de 2024, conservar tickets originales</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>2024</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>2024-06-10</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>AMAZON</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>mobiliario</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>mobiliario_y_equipamiento</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>4 bases tapizadas 120x190</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>Pedido Amazon + factura ES421LCLRAEUS</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>402-6402422-7836305</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>351.96</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t>FUERTE</t>
-        </is>
-      </c>
-      <c r="L11" t="inlineStr">
-        <is>
-          <t>Detalle de pedido con envio a Menendez Pidal; la factura visible es unitaria pero Jero confirma 4 unidades</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>2024</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>2024-06-20</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>IKEA</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>mobiliario</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>mobiliario_y_equipamiento</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>Compra tienda IKEA ticket simplificado</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>Factura simplificada SIM_691_2024/0174981</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>SIM_691_2024/0174981</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>369.21</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>FLOJO</t>
-        </is>
-      </c>
-      <c r="L12" t="inlineStr">
-        <is>
-          <t>Ticket real pero sin nombre NIF ni direccion visibles en el extracto compartido</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>2024</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>2024-06-26</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>IKEA</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>mobiliario</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>mobiliario_y_equipamiento</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>Compra IKEA con entrega a Menendez Pidal</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>Factura ESSIM24000000034880</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>1443737502</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>579.16</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>FUERTE</t>
-        </is>
-      </c>
-      <c r="L13" t="inlineStr">
-        <is>
-          <t>Direccion de envio a Menendez Pidal y detalle completo de articulos</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>2024</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>2024-07-09</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>IKEA</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>mobiliario</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>mobiliario_y_equipamiento</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>Compra tienda IKEA ticket simplificado</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>Factura simplificada SIM_691_2024/0195936</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>SIM_691_2024/0195936</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>142.21</t>
-        </is>
-      </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="K14" t="inlineStr">
-        <is>
-          <t>FLOJO</t>
-        </is>
-      </c>
-      <c r="L14" t="inlineStr">
-        <is>
-          <t>Ticket real pero sin nombre NIF ni direccion visibles en el extracto compartido</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>2024</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>2024-07-07</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>AMAZON</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>mobiliario</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>mobiliario_y_equipamiento</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>Almohadas y protectores enviado a Viator</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>Factura ES421LCLPAEUS</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>404-8694384-4720359</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>161.93</t>
-        </is>
-      </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K15" t="inlineStr">
-        <is>
-          <t>PROPIO_PERO_EXCLUIDO</t>
-        </is>
-      </c>
-      <c r="L15" t="inlineStr">
-        <is>
-          <t>Jero decide no usar en Hacienda al enviarse a Grupo Chemie Viator</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>2024</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>2024-07-08</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>AMAZON</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>mobiliario</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>mobiliario_y_equipamiento</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>Fundas de almohada enviado a Viator</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>Factura ES421LCLQAEUS</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>404-2782946-5035510</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>45.56</t>
-        </is>
-      </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K16" t="inlineStr">
-        <is>
-          <t>PROPIO_PERO_EXCLUIDO</t>
-        </is>
-      </c>
-      <c r="L16" t="inlineStr">
-        <is>
-          <t>Jero decide no usar en Hacienda al enviarse a Grupo Chemie Viator</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>2024</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>2024-07-08</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>AMAZON</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>mobiliario</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>mobiliario_y_equipamiento</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>Escobillas WC enviado a Viator</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>Factura ES421LCLOAEUS</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>404-6553842-1560302</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>10.48</t>
-        </is>
-      </c>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K17" t="inlineStr">
-        <is>
-          <t>PROPIO_PERO_EXCLUIDO</t>
-        </is>
-      </c>
-      <c r="L17" t="inlineStr">
-        <is>
-          <t>Jero decide no usar en Hacienda al enviarse a Grupo Chemie Viator</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>2024</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>2024-07-11</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>AMAZON</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>mobiliario</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>mobiliario_y_equipamiento</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>Posteres enviado a Viator</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>Factura DS-ASE-INV-ES-2024-62121755</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>404-8326125-2181120</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>18.69</t>
-        </is>
-      </c>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K18" t="inlineStr">
-        <is>
-          <t>PROPIO_PERO_EXCLUIDO</t>
-        </is>
-      </c>
-      <c r="L18" t="inlineStr">
-        <is>
-          <t>Jero decide no usar en Hacienda al enviarse a Grupo Chemie Viator</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>2024</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>2024-07-11</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>AMAZON</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>mobiliario</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>mobiliario_y_equipamiento</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>Rellenos de cojines enviado a Viator</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>Factura SIM-INV-ES-1461148515-2024-688</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>404-9365037-7246721</t>
-        </is>
-      </c>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>36.80</t>
-        </is>
-      </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K19" t="inlineStr">
-        <is>
-          <t>PROPIO_PERO_EXCLUIDO</t>
-        </is>
-      </c>
-      <c r="L19" t="inlineStr">
-        <is>
-          <t>Jero decide no usar en Hacienda al enviarse a Grupo Chemie Viator</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>2024</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>2024-07-15</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>AMAZON</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>mobiliario</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>mobiliario_y_equipamiento</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>Microondas enviado a Viator</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>Factura ES421LCLNAEUS</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>402-6883202-0465961</t>
-        </is>
-      </c>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>51.90</t>
-        </is>
-      </c>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K20" t="inlineStr">
-        <is>
-          <t>PROPIO_PERO_EXCLUIDO</t>
-        </is>
-      </c>
-      <c r="L20" t="inlineStr">
-        <is>
-          <t>Jero decide no usar en Hacienda al enviarse a Grupo Chemie Viator</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-</worksheet>
+<ns0:worksheet xmlns:ns0="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <ns0:sheetData>
+    <ns0:row r="1">
+      <ns0:c r="A1" t="inlineStr" s="1">
+        <ns0:is>
+          <ns0:t>ejercicio_devengo</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B1" t="inlineStr" s="1">
+        <ns0:is>
+          <ns0:t>fecha</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C1" t="inlineStr" s="1">
+        <ns0:is>
+          <ns0:t>proveedor</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D1" t="inlineStr" s="1">
+        <ns0:is>
+          <ns0:t>bloque</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E1" t="inlineStr" s="1">
+        <ns0:is>
+          <ns0:t>subbloque</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F1" t="inlineStr" s="1">
+        <ns0:is>
+          <ns0:t>concepto</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="G1" t="inlineStr" s="1">
+        <ns0:is>
+          <ns0:t>documento</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="H1" t="inlineStr" s="1">
+        <ns0:is>
+          <ns0:t>pedido_o_ref</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="I1" t="inlineStr" s="1">
+        <ns0:is>
+          <ns0:t>importe_total_eur</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J1" t="inlineStr" s="1">
+        <ns0:is>
+          <ns0:t>usar_hacienda</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="K1" t="inlineStr" s="1">
+        <ns0:is>
+          <ns0:t>nivel_soporte</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="L1" t="inlineStr" s="1">
+        <ns0:is>
+          <ns0:t>observaciones</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="2">
+      <ns0:c r="A2" t="inlineStr">
+        <ns0:is>
+          <ns0:t>2023</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B2" t="inlineStr">
+        <ns0:is>
+          <ns0:t>2023-11-28</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C2" t="inlineStr">
+        <ns0:is>
+          <ns0:t>OBRAMAT</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D2" t="inlineStr">
+        <ns0:is>
+          <ns0:t>reforma</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E2" t="inlineStr">
+        <ns0:is>
+          <ns0:t>obra_reforma</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F2" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Materiales reforma pedido 228131</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="G2" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Factura 003-0011-399514</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="H2" t="inlineStr">
+        <ns0:is>
+          <ns0:t>228131</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="I2" t="inlineStr">
+        <ns0:is>
+          <ns0:t>4803.37</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J2" t="inlineStr">
+        <ns0:is>
+          <ns0:t>SI</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="K2" t="inlineStr">
+        <ns0:is>
+          <ns0:t>FUERTE</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="L2" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Factura duplicada con titular NIF y direccion de Menendez Pidal; importe total TTI extraído por pdftotext de factura PDF</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="3">
+      <ns0:c r="A3" t="inlineStr">
+        <ns0:is>
+          <ns0:t>2023</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B3" t="inlineStr">
+        <ns0:is>
+          <ns0:t>2023-12-07</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C3" t="inlineStr">
+        <ns0:is>
+          <ns0:t>OBRAMAT</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D3" t="inlineStr">
+        <ns0:is>
+          <ns0:t>reforma</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E3" t="inlineStr">
+        <ns0:is>
+          <ns0:t>obra_reforma</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F3" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Materiales reforma pedido 228543</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="G3" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Factura 003-0012-404381</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="H3" t="inlineStr">
+        <ns0:is>
+          <ns0:t>228543</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="I3" t="inlineStr">
+        <ns0:is>
+          <ns0:t>161.13</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J3" t="inlineStr">
+        <ns0:is>
+          <ns0:t>SI</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="K3" t="inlineStr">
+        <ns0:is>
+          <ns0:t>FUERTE</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="L3" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Factura duplicada con titular NIF y direccion de Menendez Pidal; importe total TTI extraído por pdftotext de factura PDF</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="4">
+      <ns0:c r="A4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>2024</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>2024-01-17</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>OBRAMAT</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>reforma</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>obra_reforma</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Materiales reforma pedido 229407</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="G4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Factura 003-0001-424413</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="H4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>229407</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="I4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>1037.22</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>SI</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="K4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>FUERTE</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="L4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Factura duplicada con titular NIF y direccion de Menendez Pidal; importe total TTI extraído por pdftotext de factura PDF</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="5">
+      <ns0:c r="A5" t="inlineStr">
+        <ns0:is>
+          <ns0:t>2024</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B5" t="inlineStr">
+        <ns0:is>
+          <ns0:t>2024-02-08</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C5" t="inlineStr">
+        <ns0:is>
+          <ns0:t>OBRAMAT</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D5" t="inlineStr">
+        <ns0:is>
+          <ns0:t>reforma</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E5" t="inlineStr">
+        <ns0:is>
+          <ns0:t>obra_reforma</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F5" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Materiales reforma pedido 230379</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="G5" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Factura 003-0002-437264</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="H5" t="inlineStr">
+        <ns0:is>
+          <ns0:t>230379</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="I5" t="inlineStr">
+        <ns0:is>
+          <ns0:t>150.37</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J5" t="inlineStr">
+        <ns0:is>
+          <ns0:t>SI</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="K5" t="inlineStr">
+        <ns0:is>
+          <ns0:t>FUERTE</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="L5" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Factura duplicada con titular NIF y direccion de Menendez Pidal; importe total TTI extraído por pdftotext de factura PDF</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="6">
+      <ns0:c r="A6" t="inlineStr">
+        <ns0:is>
+          <ns0:t>2024</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B6" t="inlineStr">
+        <ns0:is>
+          <ns0:t>2024-04-15</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C6" t="inlineStr">
+        <ns0:is>
+          <ns0:t>CECOTEC</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D6" t="inlineStr">
+        <ns0:is>
+          <ns0:t>reforma</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E6" t="inlineStr">
+        <ns0:is>
+          <ns0:t>equipamiento_fijo</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F6" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Frigorifico Bolero CoolMarket Combi 250 White E</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="G6" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Factura 259006389</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="H6" t="inlineStr">
+        <ns0:is>
+          <ns0:t>256CEC-259006389</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="I6" t="inlineStr">
+        <ns0:is>
+          <ns0:t>329.00</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J6" t="inlineStr">
+        <ns0:is>
+          <ns0:t>SI</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="K6" t="inlineStr">
+        <ns0:is>
+          <ns0:t>FUERTE</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="L6" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Factura nominativa sustitutiva de simplificada; facturas sustitutivas/canje emitidas el 08/06/2026 para compras de 2024, conservar tickets originales</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="7">
+      <ns0:c r="A7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>2024</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>2024-04-19</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>CECOTEC</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>mobiliario</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>mobiliario_y_equipamiento</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Colchon Flow Viscocare 1900 120x190 unidad 1</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="G7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Factura 259006390</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="H7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>256CEC-259006390</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="I7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>119.00</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>SI</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="K7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>FUERTE</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="L7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Factura nominativa sustitutiva de simplificada; facturas sustitutivas/canje emitidas el 08/06/2026 para compras de 2024, conservar tickets originales</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="8">
+      <ns0:c r="A8" t="inlineStr">
+        <ns0:is>
+          <ns0:t>2024</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B8" t="inlineStr">
+        <ns0:is>
+          <ns0:t>2024-04-19</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C8" t="inlineStr">
+        <ns0:is>
+          <ns0:t>CECOTEC</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D8" t="inlineStr">
+        <ns0:is>
+          <ns0:t>mobiliario</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E8" t="inlineStr">
+        <ns0:is>
+          <ns0:t>mobiliario_y_equipamiento</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F8" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Colchon Flow Viscocare 1900 120x190 unidad 2</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="G8" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Factura 259006391</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="H8" t="inlineStr">
+        <ns0:is>
+          <ns0:t>256CEC-259006391</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="I8" t="inlineStr">
+        <ns0:is>
+          <ns0:t>119.00</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J8" t="inlineStr">
+        <ns0:is>
+          <ns0:t>SI</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="K8" t="inlineStr">
+        <ns0:is>
+          <ns0:t>FUERTE</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="L8" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Factura nominativa sustitutiva de simplificada; facturas sustitutivas/canje emitidas el 08/06/2026 para compras de 2024, conservar tickets originales</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="9">
+      <ns0:c r="A9" t="inlineStr">
+        <ns0:is>
+          <ns0:t>2024</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B9" t="inlineStr">
+        <ns0:is>
+          <ns0:t>2024-04-19</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C9" t="inlineStr">
+        <ns0:is>
+          <ns0:t>CECOTEC</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D9" t="inlineStr">
+        <ns0:is>
+          <ns0:t>mobiliario</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E9" t="inlineStr">
+        <ns0:is>
+          <ns0:t>mobiliario_y_equipamiento</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F9" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Colchon Flow Viscocare 1900 120x190 unidad 3</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="G9" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Factura 259006392</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="H9" t="inlineStr">
+        <ns0:is>
+          <ns0:t>256CEC-259006392</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="I9" t="inlineStr">
+        <ns0:is>
+          <ns0:t>119.00</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J9" t="inlineStr">
+        <ns0:is>
+          <ns0:t>SI</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="K9" t="inlineStr">
+        <ns0:is>
+          <ns0:t>FUERTE</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="L9" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Factura nominativa sustitutiva de simplificada; facturas sustitutivas/canje emitidas el 08/06/2026 para compras de 2024, conservar tickets originales</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="10">
+      <ns0:c r="A10" t="inlineStr">
+        <ns0:is>
+          <ns0:t>2024</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B10" t="inlineStr">
+        <ns0:is>
+          <ns0:t>2024-04-19</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C10" t="inlineStr">
+        <ns0:is>
+          <ns0:t>CECOTEC</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D10" t="inlineStr">
+        <ns0:is>
+          <ns0:t>mobiliario</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E10" t="inlineStr">
+        <ns0:is>
+          <ns0:t>mobiliario_y_equipamiento</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F10" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Colchon Flow Viscocare 1900 120x190 unidad 4</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="G10" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Factura 259006393</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="H10" t="inlineStr">
+        <ns0:is>
+          <ns0:t>256CEC-259006393</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="I10" t="inlineStr">
+        <ns0:is>
+          <ns0:t>119.00</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J10" t="inlineStr">
+        <ns0:is>
+          <ns0:t>SI</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="K10" t="inlineStr">
+        <ns0:is>
+          <ns0:t>FUERTE</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="L10" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Factura nominativa sustitutiva de simplificada; facturas sustitutivas/canje emitidas el 08/06/2026 para compras de 2024, conservar tickets originales</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="11">
+      <ns0:c r="A11" t="inlineStr">
+        <ns0:is>
+          <ns0:t>2024</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B11" t="inlineStr">
+        <ns0:is>
+          <ns0:t>2024-06-10</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C11" t="inlineStr">
+        <ns0:is>
+          <ns0:t>AMAZON</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D11" t="inlineStr">
+        <ns0:is>
+          <ns0:t>mobiliario</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E11" t="inlineStr">
+        <ns0:is>
+          <ns0:t>mobiliario_y_equipamiento</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F11" t="inlineStr">
+        <ns0:is>
+          <ns0:t>4 bases tapizadas 120x190</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="G11" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Pedido Amazon + factura ES421LCLRAEUS</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="H11" t="inlineStr">
+        <ns0:is>
+          <ns0:t>402-6402422-7836305</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="I11" t="inlineStr">
+        <ns0:is>
+          <ns0:t>351.96</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J11" t="inlineStr">
+        <ns0:is>
+          <ns0:t>SI</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="K11" t="inlineStr">
+        <ns0:is>
+          <ns0:t>FUERTE</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="L11" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Detalle de pedido con envio a Menendez Pidal; la factura visible es unitaria pero Jero confirma 4 unidades</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="12">
+      <ns0:c r="A12" t="inlineStr">
+        <ns0:is>
+          <ns0:t>2024</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B12" t="inlineStr">
+        <ns0:is>
+          <ns0:t>2024-06-20</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C12" t="inlineStr">
+        <ns0:is>
+          <ns0:t>IKEA</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D12" t="inlineStr">
+        <ns0:is>
+          <ns0:t>mobiliario</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E12" t="inlineStr">
+        <ns0:is>
+          <ns0:t>mobiliario_y_equipamiento</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F12" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Compra tienda IKEA ticket simplificado</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="G12" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Factura simplificada SIM_691_2024/0174981</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="H12" t="inlineStr">
+        <ns0:is>
+          <ns0:t>SIM_691_2024/0174981</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="I12" t="inlineStr">
+        <ns0:is>
+          <ns0:t>369.21</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J12" t="inlineStr">
+        <ns0:is>
+          <ns0:t>PENDIENTE</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="K12" t="inlineStr">
+        <ns0:is>
+          <ns0:t>FLOJO</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="L12" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Ticket real pero sin nombre NIF ni direccion visibles en el extracto compartido</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="13">
+      <ns0:c r="A13" t="inlineStr">
+        <ns0:is>
+          <ns0:t>2024</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B13" t="inlineStr">
+        <ns0:is>
+          <ns0:t>2024-06-26</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C13" t="inlineStr">
+        <ns0:is>
+          <ns0:t>IKEA</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D13" t="inlineStr">
+        <ns0:is>
+          <ns0:t>mobiliario</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E13" t="inlineStr">
+        <ns0:is>
+          <ns0:t>mobiliario_y_equipamiento</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F13" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Compra IKEA con entrega a Menendez Pidal</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="G13" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Factura ESSIM24000000034880</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="H13" t="inlineStr">
+        <ns0:is>
+          <ns0:t>1443737502</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="I13" t="inlineStr">
+        <ns0:is>
+          <ns0:t>579.16</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J13" t="inlineStr">
+        <ns0:is>
+          <ns0:t>SI</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="K13" t="inlineStr">
+        <ns0:is>
+          <ns0:t>FUERTE</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="L13" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Direccion de envio a Menendez Pidal y detalle completo de articulos</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="14">
+      <ns0:c r="A14" t="inlineStr">
+        <ns0:is>
+          <ns0:t>2024</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B14" t="inlineStr">
+        <ns0:is>
+          <ns0:t>2024-07-09</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C14" t="inlineStr">
+        <ns0:is>
+          <ns0:t>IKEA</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D14" t="inlineStr">
+        <ns0:is>
+          <ns0:t>mobiliario</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E14" t="inlineStr">
+        <ns0:is>
+          <ns0:t>mobiliario_y_equipamiento</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F14" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Compra tienda IKEA ticket simplificado</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="G14" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Factura simplificada SIM_691_2024/0195936</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="H14" t="inlineStr">
+        <ns0:is>
+          <ns0:t>SIM_691_2024/0195936</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="I14" t="inlineStr">
+        <ns0:is>
+          <ns0:t>142.21</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J14" t="inlineStr">
+        <ns0:is>
+          <ns0:t>PENDIENTE</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="K14" t="inlineStr">
+        <ns0:is>
+          <ns0:t>FLOJO</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="L14" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Ticket real pero sin nombre NIF ni direccion visibles en el extracto compartido</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="15">
+      <ns0:c r="A15" t="inlineStr">
+        <ns0:is>
+          <ns0:t>2024</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B15" t="inlineStr">
+        <ns0:is>
+          <ns0:t>2024-07-07</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C15" t="inlineStr">
+        <ns0:is>
+          <ns0:t>AMAZON</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D15" t="inlineStr">
+        <ns0:is>
+          <ns0:t>mobiliario</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E15" t="inlineStr">
+        <ns0:is>
+          <ns0:t>mobiliario_y_equipamiento</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F15" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Almohadas y protectores enviado a Viator</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="G15" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Factura ES421LCLPAEUS</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="H15" t="inlineStr">
+        <ns0:is>
+          <ns0:t>404-8694384-4720359</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="I15" t="inlineStr">
+        <ns0:is>
+          <ns0:t>161.93</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J15" t="inlineStr">
+        <ns0:is>
+          <ns0:t>NO</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="K15" t="inlineStr">
+        <ns0:is>
+          <ns0:t>PROPIO_PERO_EXCLUIDO</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="L15" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Jero decide no usar en Hacienda al enviarse a Grupo Chemie Viator</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="16">
+      <ns0:c r="A16" t="inlineStr">
+        <ns0:is>
+          <ns0:t>2024</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B16" t="inlineStr">
+        <ns0:is>
+          <ns0:t>2024-07-08</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C16" t="inlineStr">
+        <ns0:is>
+          <ns0:t>AMAZON</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D16" t="inlineStr">
+        <ns0:is>
+          <ns0:t>mobiliario</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E16" t="inlineStr">
+        <ns0:is>
+          <ns0:t>mobiliario_y_equipamiento</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F16" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Fundas de almohada enviado a Viator</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="G16" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Factura ES421LCLQAEUS</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="H16" t="inlineStr">
+        <ns0:is>
+          <ns0:t>404-2782946-5035510</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="I16" t="inlineStr">
+        <ns0:is>
+          <ns0:t>45.56</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J16" t="inlineStr">
+        <ns0:is>
+          <ns0:t>NO</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="K16" t="inlineStr">
+        <ns0:is>
+          <ns0:t>PROPIO_PERO_EXCLUIDO</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="L16" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Jero decide no usar en Hacienda al enviarse a Grupo Chemie Viator</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="17">
+      <ns0:c r="A17" t="inlineStr">
+        <ns0:is>
+          <ns0:t>2024</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B17" t="inlineStr">
+        <ns0:is>
+          <ns0:t>2024-07-08</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C17" t="inlineStr">
+        <ns0:is>
+          <ns0:t>AMAZON</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D17" t="inlineStr">
+        <ns0:is>
+          <ns0:t>mobiliario</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E17" t="inlineStr">
+        <ns0:is>
+          <ns0:t>mobiliario_y_equipamiento</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F17" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Escobillas WC enviado a Viator</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="G17" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Factura ES421LCLOAEUS</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="H17" t="inlineStr">
+        <ns0:is>
+          <ns0:t>404-6553842-1560302</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="I17" t="inlineStr">
+        <ns0:is>
+          <ns0:t>10.48</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J17" t="inlineStr">
+        <ns0:is>
+          <ns0:t>NO</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="K17" t="inlineStr">
+        <ns0:is>
+          <ns0:t>PROPIO_PERO_EXCLUIDO</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="L17" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Jero decide no usar en Hacienda al enviarse a Grupo Chemie Viator</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="18">
+      <ns0:c r="A18" t="inlineStr">
+        <ns0:is>
+          <ns0:t>2024</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B18" t="inlineStr">
+        <ns0:is>
+          <ns0:t>2024-07-11</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C18" t="inlineStr">
+        <ns0:is>
+          <ns0:t>AMAZON</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D18" t="inlineStr">
+        <ns0:is>
+          <ns0:t>mobiliario</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E18" t="inlineStr">
+        <ns0:is>
+          <ns0:t>mobiliario_y_equipamiento</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F18" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Posteres enviado a Viator</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="G18" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Factura DS-ASE-INV-ES-2024-62121755</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="H18" t="inlineStr">
+        <ns0:is>
+          <ns0:t>404-8326125-2181120</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="I18" t="inlineStr">
+        <ns0:is>
+          <ns0:t>18.69</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J18" t="inlineStr">
+        <ns0:is>
+          <ns0:t>NO</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="K18" t="inlineStr">
+        <ns0:is>
+          <ns0:t>PROPIO_PERO_EXCLUIDO</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="L18" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Jero decide no usar en Hacienda al enviarse a Grupo Chemie Viator</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="19">
+      <ns0:c r="A19" t="inlineStr">
+        <ns0:is>
+          <ns0:t>2024</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B19" t="inlineStr">
+        <ns0:is>
+          <ns0:t>2024-07-11</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C19" t="inlineStr">
+        <ns0:is>
+          <ns0:t>AMAZON</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D19" t="inlineStr">
+        <ns0:is>
+          <ns0:t>mobiliario</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E19" t="inlineStr">
+        <ns0:is>
+          <ns0:t>mobiliario_y_equipamiento</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F19" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Rellenos de cojines enviado a Viator</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="G19" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Factura SIM-INV-ES-1461148515-2024-688</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="H19" t="inlineStr">
+        <ns0:is>
+          <ns0:t>404-9365037-7246721</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="I19" t="inlineStr">
+        <ns0:is>
+          <ns0:t>36.80</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J19" t="inlineStr">
+        <ns0:is>
+          <ns0:t>NO</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="K19" t="inlineStr">
+        <ns0:is>
+          <ns0:t>PROPIO_PERO_EXCLUIDO</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="L19" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Jero decide no usar en Hacienda al enviarse a Grupo Chemie Viator</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="20">
+      <ns0:c r="A20" t="inlineStr">
+        <ns0:is>
+          <ns0:t>2024</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B20" t="inlineStr">
+        <ns0:is>
+          <ns0:t>2024-07-15</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C20" t="inlineStr">
+        <ns0:is>
+          <ns0:t>AMAZON</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D20" t="inlineStr">
+        <ns0:is>
+          <ns0:t>mobiliario</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E20" t="inlineStr">
+        <ns0:is>
+          <ns0:t>mobiliario_y_equipamiento</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F20" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Microondas enviado a Viator</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="G20" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Factura ES421LCLNAEUS</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="H20" t="inlineStr">
+        <ns0:is>
+          <ns0:t>402-6883202-0465961</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="I20" t="inlineStr">
+        <ns0:is>
+          <ns0:t>51.90</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J20" t="inlineStr">
+        <ns0:is>
+          <ns0:t>NO</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="K20" t="inlineStr">
+        <ns0:is>
+          <ns0:t>PROPIO_PERO_EXCLUIDO</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="L20" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Jero decide no usar en Hacienda al enviarse a Grupo Chemie Viator</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="21">
+      <ns0:c r="A21" t="inlineStr">
+        <ns0:is>
+          <ns0:t>2023</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B21" t="inlineStr">
+        <ns0:is>
+          <ns0:t>2023-11-27</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C21" t="inlineStr">
+        <ns0:is>
+          <ns0:t>OBRAMAT</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D21" t="inlineStr">
+        <ns0:is>
+          <ns0:t>reforma</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E21" t="inlineStr">
+        <ns0:is>
+          <ns0:t>anticipo_pedido</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F21" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Anticipo pedido 228131</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="G21" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Factura 003-0011-398765</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="H21" t="inlineStr">
+        <ns0:is>
+          <ns0:t>228131</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="I21" t="inlineStr">
+        <ns0:is>
+          <ns0:t>4803.37</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J21" t="inlineStr">
+        <ns0:is>
+          <ns0:t>NO_SEPARADO</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="K21" t="inlineStr">
+        <ns0:is>
+          <ns0:t>FUERTE</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="L21" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Factura nominativa real de anticipo. Mismo TTI que la factura de entrega 003-0011-399514; no sumar aparte para evitar duplicidad, usar solo como refuerzo documental del pedido 228131.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="22">
+      <ns0:c r="A22" t="inlineStr">
+        <ns0:is>
+          <ns0:t>2023</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B22" t="inlineStr">
+        <ns0:is>
+          <ns0:t>2023-12-07</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C22" t="inlineStr">
+        <ns0:is>
+          <ns0:t>OBRAMAT</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D22" t="inlineStr">
+        <ns0:is>
+          <ns0:t>reforma</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E22" t="inlineStr">
+        <ns0:is>
+          <ns0:t>anticipo_pedido</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F22" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Anticipo pedido 228543</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="G22" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Factura 003-0012-404208</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="H22" t="inlineStr">
+        <ns0:is>
+          <ns0:t>228543</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="I22" t="inlineStr">
+        <ns0:is>
+          <ns0:t>161.13</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J22" t="inlineStr">
+        <ns0:is>
+          <ns0:t>NO_SEPARADO</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="K22" t="inlineStr">
+        <ns0:is>
+          <ns0:t>FUERTE</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="L22" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Factura nominativa real de anticipo. Mismo TTI que la factura de entrega 003-0012-404381; no sumar aparte para evitar duplicidad, usar solo como refuerzo documental del pedido 228543.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="23">
+      <ns0:c r="A23" t="inlineStr">
+        <ns0:is>
+          <ns0:t>2024</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B23" t="inlineStr">
+        <ns0:is>
+          <ns0:t>2024-01-12</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C23" t="inlineStr">
+        <ns0:is>
+          <ns0:t>OBRAMAT</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D23" t="inlineStr">
+        <ns0:is>
+          <ns0:t>reforma</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E23" t="inlineStr">
+        <ns0:is>
+          <ns0:t>anticipo_pedido</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F23" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Anticipo pedido 229407</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="G23" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Factura 003-0001-421861</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="H23" t="inlineStr">
+        <ns0:is>
+          <ns0:t>229407</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="I23" t="inlineStr">
+        <ns0:is>
+          <ns0:t>1037.22</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J23" t="inlineStr">
+        <ns0:is>
+          <ns0:t>NO_SEPARADO</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="K23" t="inlineStr">
+        <ns0:is>
+          <ns0:t>FUERTE</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="L23" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Factura nominativa real de anticipo. Mismo TTI que la factura de entrega 003-0001-424413; no sumar aparte para evitar duplicidad, usar solo como refuerzo documental del pedido 229407.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="24">
+      <ns0:c r="A24" t="inlineStr">
+        <ns0:is>
+          <ns0:t>2024</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B24" t="inlineStr">
+        <ns0:is>
+          <ns0:t>2024-02-07</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C24" t="inlineStr">
+        <ns0:is>
+          <ns0:t>OBRAMAT</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D24" t="inlineStr">
+        <ns0:is>
+          <ns0:t>reforma</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E24" t="inlineStr">
+        <ns0:is>
+          <ns0:t>anticipo_pedido</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F24" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Anticipo pedido 230379</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="G24" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Factura 003-0002-436986</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="H24" t="inlineStr">
+        <ns0:is>
+          <ns0:t>230379</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="I24" t="inlineStr">
+        <ns0:is>
+          <ns0:t>150.37</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J24" t="inlineStr">
+        <ns0:is>
+          <ns0:t>NO_SEPARADO</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="K24" t="inlineStr">
+        <ns0:is>
+          <ns0:t>FUERTE</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="L24" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Factura nominativa real de anticipo. Mismo TTI que la factura de entrega 003-0002-437264; no sumar aparte para evitar duplicidad, usar solo como refuerzo documental del pedido 230379.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="25">
+      <ns0:c r="A25" t="inlineStr">
+        <ns0:is>
+          <ns0:t>2023</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B25" t="inlineStr">
+        <ns0:is>
+          <ns0:t>2023-12-07</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C25" t="inlineStr">
+        <ns0:is>
+          <ns0:t>OBRAMAT</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D25" t="inlineStr">
+        <ns0:is>
+          <ns0:t>reforma</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E25" t="inlineStr">
+        <ns0:is>
+          <ns0:t>materiales_satélite</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F25" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Compra autónoma adicional Obramat</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="G25" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Factura 003-0012-404213</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="H25" t="inlineStr">
+        <ns0:is>
+          <ns0:t>404213</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="I25" t="inlineStr">
+        <ns0:is>
+          <ns0:t>80.19</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J25" t="inlineStr">
+        <ns0:is>
+          <ns0:t>PENDIENTE</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="K25" t="inlineStr">
+        <ns0:is>
+          <ns0:t>FUERTE</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="L25" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Factura nominativa real no integrada en los 4 pedidos principales. Compra separada, plausible para la obra, pendiente de decidir si se incorpora al núcleo de reforma.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="26">
+      <ns0:c r="A26" t="inlineStr">
+        <ns0:is>
+          <ns0:t>2023</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B26" t="inlineStr">
+        <ns0:is>
+          <ns0:t>2023-12-13</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C26" t="inlineStr">
+        <ns0:is>
+          <ns0:t>OBRAMAT</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D26" t="inlineStr">
+        <ns0:is>
+          <ns0:t>reforma</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E26" t="inlineStr">
+        <ns0:is>
+          <ns0:t>materiales_satélite</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F26" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Compra autónoma adicional Obramat</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="G26" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Factura 003-0012-407792</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="H26" t="inlineStr">
+        <ns0:is>
+          <ns0:t>407792</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="I26" t="inlineStr">
+        <ns0:is>
+          <ns0:t>21.90</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J26" t="inlineStr">
+        <ns0:is>
+          <ns0:t>PENDIENTE</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="K26" t="inlineStr">
+        <ns0:is>
+          <ns0:t>FUERTE</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="L26" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Factura nominativa real no integrada en los 4 pedidos principales. Compra pequeña de escayola, plausible para la obra.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="27">
+      <ns0:c r="A27" t="inlineStr">
+        <ns0:is>
+          <ns0:t>2024</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B27" t="inlineStr">
+        <ns0:is>
+          <ns0:t>2024-03-05</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C27" t="inlineStr">
+        <ns0:is>
+          <ns0:t>OBRAMAT</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D27" t="inlineStr">
+        <ns0:is>
+          <ns0:t>reforma</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E27" t="inlineStr">
+        <ns0:is>
+          <ns0:t>materiales_satélite</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F27" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Compra autónoma adicional Obramat</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="G27" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Factura 003-0003-452497</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="H27" t="inlineStr">
+        <ns0:is>
+          <ns0:t>452497</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="I27" t="inlineStr">
+        <ns0:is>
+          <ns0:t>39.53</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J27" t="inlineStr">
+        <ns0:is>
+          <ns0:t>PENDIENTE</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="K27" t="inlineStr">
+        <ns0:is>
+          <ns0:t>FUERTE</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="L27" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Factura nominativa real no integrada en los 4 pedidos principales. Material eléctrico/plaqueado, plausible para remates de obra.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="28">
+      <ns0:c r="A28" t="inlineStr">
+        <ns0:is>
+          <ns0:t>2024</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B28" t="inlineStr">
+        <ns0:is>
+          <ns0:t>2024-03-05</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C28" t="inlineStr">
+        <ns0:is>
+          <ns0:t>OBRAMAT</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D28" t="inlineStr">
+        <ns0:is>
+          <ns0:t>reforma</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E28" t="inlineStr">
+        <ns0:is>
+          <ns0:t>materiales_satélite</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F28" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Compra autónoma adicional Obramat</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="G28" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Factura 003-0003-452516</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="H28" t="inlineStr">
+        <ns0:is>
+          <ns0:t>452516</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="I28" t="inlineStr">
+        <ns0:is>
+          <ns0:t>135.00</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J28" t="inlineStr">
+        <ns0:is>
+          <ns0:t>PENDIENTE</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="K28" t="inlineStr">
+        <ns0:is>
+          <ns0:t>FUERTE</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="L28" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Factura nominativa real no integrada en los 4 pedidos principales. Mampara, muy conectable con la reforma del baño.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+  </ns0:sheetData>
+</ns0:worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>